<commit_message>
Math: lock option B prices (100/300/600x) and update docs
Double starts the rewind multiplier at x3, Director gets 13 free spins.
Regenerated workbook and MATH.md tables for the new modes.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XbWfUAM6YhZVGBMbPhdX3o
</commit_message>
<xml_diff>
--- a/math/LateFeeVideo_math_v0.2.xlsx
+++ b/math/LateFeeVideo_math_v0.2.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1427" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1427" uniqueCount="121">
   <si>
     <t xml:space="preserve">Late Fee Video — режимы (прототип JS, естественный RTP до оптимизации весов)</t>
   </si>
@@ -271,6 +271,9 @@
   </si>
   <si>
     <t xml:space="preserve">Buy «Двойной сеанс»: стартовый множитель</t>
+  </si>
+  <si>
+    <t xml:space="preserve">×3</t>
   </si>
   <si>
     <t xml:space="preserve">Buy «Двойной сеанс»: гарантированный REW</t>
@@ -1067,29 +1070,29 @@
         <v>500000</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>260</v>
+        <v>300</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>249.99</v>
+        <v>294.3</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">E8/D8</f>
-        <v>0.9615</v>
+        <v>0.981</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>0.96</v>
       </c>
       <c r="H8" s="5" t="n">
         <f aca="false">F8-G8</f>
-        <v>0.00150000000000006</v>
+        <v>0.021</v>
       </c>
       <c r="I8" s="5" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
       <c r="J8" s="5" t="n">
-        <f aca="false">0.9615</f>
-        <v>0.9615</v>
+        <f aca="false">0.981</f>
+        <v>0.981</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>1</v>
@@ -1098,10 +1101,10 @@
         <v>1</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>250</v>
+        <v>294.29</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>1.12</v>
+        <v>1.07</v>
       </c>
       <c r="O8" s="2" t="n">
         <v>11817</v>
@@ -1125,29 +1128,29 @@
         <v>500000</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>570</v>
+        <v>600</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>547.086</v>
+        <v>606.42</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">E9/D9</f>
-        <v>0.9598</v>
+        <v>1.0107</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>0.96</v>
       </c>
       <c r="H9" s="5" t="n">
         <f aca="false">F9-G9</f>
-        <v>-0.000199999999999978</v>
+        <v>0.0507</v>
       </c>
       <c r="I9" s="5" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
       <c r="J9" s="5" t="n">
-        <f aca="false">0.9598</f>
-        <v>0.9598</v>
+        <f aca="false">1.0107</f>
+        <v>1.0107</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>1</v>
@@ -1156,10 +1159,10 @@
         <v>1</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>547.09</v>
+        <v>606.41</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.9</v>
+        <v>0.94</v>
       </c>
       <c r="O9" s="2" t="n">
         <v>15000</v>
@@ -1766,39 +1769,39 @@
         <v>80</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B13" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1822,12 +1825,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1835,19 +1838,19 @@
         <v>31</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2072,7 +2075,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>0</v>
@@ -2092,7 +2095,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>2</v>
@@ -2112,7 +2115,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>0</v>
@@ -2132,7 +2135,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B19" s="7" t="n">
         <f aca="false">SUM(B5:B18)</f>
@@ -2157,7 +2160,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2165,19 +2168,19 @@
         <v>31</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2402,7 +2405,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>0</v>
@@ -2422,7 +2425,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>4</v>
@@ -2442,7 +2445,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>0</v>
@@ -2462,7 +2465,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B37" s="7" t="n">
         <f aca="false">SUM(B23:B36)</f>
@@ -2487,7 +2490,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2495,19 +2498,19 @@
         <v>31</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2732,7 +2735,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>0</v>
@@ -2752,7 +2755,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>2</v>
@@ -2772,7 +2775,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>0</v>
@@ -2792,7 +2795,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B55" s="7" t="n">
         <f aca="false">SUM(B41:B54)</f>
@@ -2836,22 +2839,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2859,7 +2862,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>58</v>
@@ -2908,7 +2911,7 @@
         <v>58</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F4" s="0" t="s">
         <v>44</v>
@@ -2945,7 +2948,7 @@
         <v>42</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E6" s="0" t="s">
         <v>46</v>
@@ -2965,7 +2968,7 @@
         <v>52</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E7" s="0" t="s">
         <v>48</v>
@@ -3105,7 +3108,7 @@
         <v>58</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E14" s="0" t="s">
         <v>52</v>
@@ -3131,7 +3134,7 @@
         <v>58</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3145,7 +3148,7 @@
         <v>58</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E16" s="0" t="s">
         <v>58</v>
@@ -3188,7 +3191,7 @@
         <v>48</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F18" s="0" t="s">
         <v>52</v>
@@ -3439,10 +3442,10 @@
         <v>29</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D31" s="0" t="s">
         <v>54</v>
@@ -3465,7 +3468,7 @@
         <v>60</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E32" s="0" t="s">
         <v>56</v>
@@ -3505,10 +3508,10 @@
         <v>46</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F34" s="0" t="s">
         <v>42</v>
@@ -3528,7 +3531,7 @@
         <v>56</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F35" s="0" t="s">
         <v>42</v>
@@ -3582,7 +3585,7 @@
         <v>50</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D38" s="0" t="s">
         <v>52</v>
@@ -3708,7 +3711,7 @@
         <v>60</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F44" s="0" t="s">
         <v>54</v>
@@ -3725,7 +3728,7 @@
         <v>54</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E45" s="0" t="s">
         <v>46</v>
@@ -3742,7 +3745,7 @@
         <v>60</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D46" s="0" t="s">
         <v>56</v>
@@ -3782,13 +3785,13 @@
         <v>46</v>
       </c>
       <c r="C48" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="D48" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="E48" s="0" t="s">
         <v>96</v>
-      </c>
-      <c r="D48" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="E48" s="0" t="s">
-        <v>95</v>
       </c>
       <c r="F48" s="0" t="s">
         <v>44</v>
@@ -3802,13 +3805,13 @@
         <v>40</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D49" s="0" t="s">
         <v>50</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F49" s="0" t="s">
         <v>58</v>
@@ -3962,7 +3965,7 @@
         <v>60</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D57" s="0" t="s">
         <v>58</v>
@@ -4042,7 +4045,7 @@
         <v>48</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D61" s="0" t="s">
         <v>60</v>
@@ -4165,7 +4168,7 @@
         <v>44</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E67" s="0" t="s">
         <v>56</v>
@@ -4291,7 +4294,7 @@
         <v>56</v>
       </c>
       <c r="F73" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4328,7 +4331,7 @@
         <v>60</v>
       </c>
       <c r="E75" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F75" s="0" t="s">
         <v>42</v>
@@ -4475,7 +4478,7 @@
         <v>82</v>
       </c>
       <c r="C84" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D84" s="0" t="s">
         <v>54</v>
@@ -4505,22 +4508,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4594,7 +4597,7 @@
         <v>48</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E5" s="0" t="s">
         <v>58</v>
@@ -4614,7 +4617,7 @@
         <v>48</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E6" s="0" t="s">
         <v>58</v>
@@ -4631,7 +4634,7 @@
         <v>50</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D7" s="0" t="s">
         <v>50</v>
@@ -4660,7 +4663,7 @@
         <v>48</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4717,7 +4720,7 @@
         <v>58</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F11" s="0" t="s">
         <v>58</v>
@@ -4731,7 +4734,7 @@
         <v>54</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D12" s="0" t="s">
         <v>44</v>
@@ -4740,7 +4743,7 @@
         <v>46</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4831,7 +4834,7 @@
         <v>60</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D17" s="0" t="s">
         <v>54</v>
@@ -4854,7 +4857,7 @@
         <v>58</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E18" s="0" t="s">
         <v>60</v>
@@ -4897,7 +4900,7 @@
         <v>44</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F20" s="0" t="s">
         <v>44</v>
@@ -4940,7 +4943,7 @@
         <v>60</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4974,7 +4977,7 @@
         <v>48</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E24" s="0" t="s">
         <v>48</v>
@@ -5014,13 +5017,13 @@
         <v>58</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E26" s="0" t="s">
         <v>58</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5097,10 +5100,10 @@
         <v>52</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5117,7 +5120,7 @@
         <v>48</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F31" s="0" t="s">
         <v>42</v>
@@ -5197,7 +5200,7 @@
         <v>42</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F35" s="0" t="s">
         <v>60</v>
@@ -5217,7 +5220,7 @@
         <v>48</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F36" s="0" t="s">
         <v>54</v>
@@ -5231,7 +5234,7 @@
         <v>46</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D37" s="0" t="s">
         <v>50</v>
@@ -5251,7 +5254,7 @@
         <v>50</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D38" s="0" t="s">
         <v>48</v>
@@ -5294,7 +5297,7 @@
         <v>46</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E40" s="0" t="s">
         <v>50</v>
@@ -5331,7 +5334,7 @@
         <v>60</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D42" s="0" t="s">
         <v>56</v>
@@ -5374,7 +5377,7 @@
         <v>54</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E44" s="0" t="s">
         <v>46</v>
@@ -5397,7 +5400,7 @@
         <v>54</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F45" s="0" t="s">
         <v>52</v>
@@ -5431,13 +5434,13 @@
         <v>42</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D47" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="E47" s="0" t="s">
         <v>96</v>
-      </c>
-      <c r="E47" s="0" t="s">
-        <v>95</v>
       </c>
       <c r="F47" s="0" t="s">
         <v>48</v>
@@ -5471,13 +5474,13 @@
         <v>56</v>
       </c>
       <c r="C49" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="D49" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="E49" s="0" t="s">
         <v>96</v>
-      </c>
-      <c r="D49" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="E49" s="0" t="s">
-        <v>95</v>
       </c>
       <c r="F49" s="0" t="s">
         <v>50</v>
@@ -5497,10 +5500,10 @@
         <v>44</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F50" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5511,7 +5514,7 @@
         <v>46</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D51" s="0" t="s">
         <v>60</v>
@@ -5614,13 +5617,13 @@
         <v>50</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E56" s="0" t="s">
         <v>42</v>
       </c>
       <c r="F56" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5671,7 +5674,7 @@
         <v>60</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D59" s="0" t="s">
         <v>50</v>
@@ -5694,7 +5697,7 @@
         <v>42</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E60" s="0" t="s">
         <v>58</v>
@@ -5708,7 +5711,7 @@
         <v>59</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C61" s="0" t="s">
         <v>50</v>
@@ -5768,16 +5771,16 @@
         <v>62</v>
       </c>
       <c r="B64" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C64" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="D64" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="E64" s="0" t="s">
         <v>96</v>
-      </c>
-      <c r="C64" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="D64" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="E64" s="0" t="s">
-        <v>95</v>
       </c>
       <c r="F64" s="0" t="s">
         <v>48</v>
@@ -5817,7 +5820,7 @@
         <v>56</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F66" s="0" t="s">
         <v>60</v>
@@ -5851,10 +5854,10 @@
         <v>58</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E68" s="0" t="s">
         <v>58</v>
@@ -5977,7 +5980,7 @@
         <v>48</v>
       </c>
       <c r="F74" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5985,7 +5988,7 @@
         <v>73</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D75" s="0" t="s">
         <v>54</v>
@@ -6101,7 +6104,7 @@
         <v>54</v>
       </c>
       <c r="D82" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E82" s="0" t="s">
         <v>48</v>
@@ -6142,22 +6145,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6168,13 +6171,13 @@
         <v>42</v>
       </c>
       <c r="C2" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="0" t="s">
         <v>96</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>95</v>
       </c>
       <c r="F2" s="0" t="s">
         <v>54</v>
@@ -6214,7 +6217,7 @@
         <v>52</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F4" s="0" t="s">
         <v>50</v>
@@ -6268,7 +6271,7 @@
         <v>52</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D7" s="0" t="s">
         <v>58</v>
@@ -6288,7 +6291,7 @@
         <v>60</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D8" s="0" t="s">
         <v>58</v>
@@ -6351,7 +6354,7 @@
         <v>44</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E11" s="0" t="s">
         <v>58</v>
@@ -6394,7 +6397,7 @@
         <v>50</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F13" s="0" t="s">
         <v>60</v>
@@ -6468,7 +6471,7 @@
         <v>50</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D17" s="0" t="s">
         <v>48</v>
@@ -6571,7 +6574,7 @@
         <v>54</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E22" s="0" t="s">
         <v>60</v>
@@ -6645,10 +6648,10 @@
         <v>24</v>
       </c>
       <c r="B26" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" s="0" t="s">
         <v>96</v>
-      </c>
-      <c r="C26" s="0" t="s">
-        <v>95</v>
       </c>
       <c r="D26" s="0" t="s">
         <v>56</v>
@@ -6677,7 +6680,7 @@
         <v>40</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6745,7 +6748,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C31" s="0" t="s">
         <v>54</v>
@@ -6754,7 +6757,7 @@
         <v>44</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F31" s="0" t="s">
         <v>60</v>
@@ -6768,10 +6771,10 @@
         <v>44</v>
       </c>
       <c r="C32" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="D32" s="0" t="s">
         <v>96</v>
-      </c>
-      <c r="D32" s="0" t="s">
-        <v>95</v>
       </c>
       <c r="E32" s="0" t="s">
         <v>60</v>
@@ -6931,7 +6934,7 @@
         <v>54</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E40" s="0" t="s">
         <v>48</v>
@@ -6951,7 +6954,7 @@
         <v>46</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E41" s="0" t="s">
         <v>48</v>
@@ -7045,7 +7048,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C46" s="0" t="s">
         <v>42</v>
@@ -7054,7 +7057,7 @@
         <v>54</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F46" s="0" t="s">
         <v>40</v>
@@ -7097,7 +7100,7 @@
         <v>56</v>
       </c>
       <c r="F48" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7134,7 +7137,7 @@
         <v>48</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F50" s="0" t="s">
         <v>52</v>
@@ -7188,7 +7191,7 @@
         <v>40</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D53" s="0" t="s">
         <v>60</v>
@@ -7225,7 +7228,7 @@
         <v>53</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C55" s="0" t="s">
         <v>58</v>
@@ -7277,7 +7280,7 @@
         <v>44</v>
       </c>
       <c r="F57" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7314,7 +7317,7 @@
         <v>60</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F59" s="0" t="s">
         <v>58</v>
@@ -7371,7 +7374,7 @@
         <v>46</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E62" s="0" t="s">
         <v>52</v>
@@ -7411,7 +7414,7 @@
         <v>60</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E64" s="0" t="s">
         <v>52</v>
@@ -7434,7 +7437,7 @@
         <v>52</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F65" s="0" t="s">
         <v>60</v>
@@ -7468,10 +7471,10 @@
         <v>60</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E67" s="0" t="s">
         <v>56</v>
@@ -7528,13 +7531,13 @@
         <v>56</v>
       </c>
       <c r="C70" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="D70" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="D70" s="0" t="s">
-        <v>95</v>
-      </c>
       <c r="E70" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F70" s="0" t="s">
         <v>46</v>
@@ -7548,7 +7551,7 @@
         <v>56</v>
       </c>
       <c r="C71" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D71" s="0" t="s">
         <v>42</v>
@@ -7614,7 +7617,7 @@
         <v>56</v>
       </c>
       <c r="E74" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F74" s="0" t="s">
         <v>58</v>
@@ -7631,7 +7634,7 @@
         <v>60</v>
       </c>
       <c r="D75" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E75" s="0" t="s">
         <v>60</v>
@@ -7788,7 +7791,7 @@
         <v>58</v>
       </c>
       <c r="F83" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7903,25 +7906,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8352,12 +8355,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>20</v>
@@ -8377,7 +8380,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">1-SUM(B5:B16)</f>
@@ -8397,12 +8400,12 @@
       </c>
       <c r="F4" s="9" t="n">
         <f aca="false">1-SUM(F5:F16)</f>
-        <v>0.00141000000000002</v>
+        <v>0.000813999999999981</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>0.05138495</v>
@@ -8417,12 +8420,12 @@
         <v>0.000574</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>4.8E-005</v>
+        <v>8.2E-005</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B6" s="9" t="n">
         <v>0.07276295</v>
@@ -8437,12 +8440,12 @@
         <v>0.000726</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>5.6E-005</v>
+        <v>0.000128</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>0.07365195</v>
@@ -8454,15 +8457,15 @@
         <v>0.025826</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.0016</v>
+        <v>0.001086</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>9.2E-005</v>
+        <v>0.000198</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>0.02183685</v>
@@ -8474,15 +8477,15 @@
         <v>0.063894</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.00582</v>
+        <v>0.003212</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>0.000458</v>
+        <v>0.000346</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B9" s="9" t="n">
         <v>0.00676245</v>
@@ -8494,15 +8497,15 @@
         <v>0.13718</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.022254</v>
+        <v>0.012586</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>0.001382</v>
+        <v>0.001104</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>0.0023518</v>
@@ -8514,15 +8517,15 @@
         <v>0.275128</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>0.104654</v>
+        <v>0.069646</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.010322</v>
+        <v>0.008084</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>0.00087855</v>
@@ -8534,15 +8537,15 @@
         <v>0.20848</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>0.18259</v>
+        <v>0.14879</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>0.040352</v>
+        <v>0.031526</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B12" s="9" t="n">
         <v>0.00098085</v>
@@ -8554,15 +8557,15 @@
         <v>0.254648</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>0.557794</v>
+        <v>0.603932</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>0.55236</v>
+        <v>0.510332</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B13" s="9" t="n">
         <v>7.705E-005</v>
@@ -8574,15 +8577,15 @@
         <v>0.020268</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>0.094354</v>
+        <v>0.12061</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>0.26984</v>
+        <v>0.295516</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B14" s="9" t="n">
         <v>1.375E-005</v>
@@ -8594,15 +8597,15 @@
         <v>0.003712</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>0.025548</v>
+        <v>0.03472</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>0.122984</v>
+        <v>0.150802</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B15" s="9" t="n">
         <v>0</v>
@@ -8614,15 +8617,15 @@
         <v>0</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>7.6E-005</v>
+        <v>0.000108</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>0.000688</v>
+        <v>0.00106</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B16" s="9" t="n">
         <v>0</v>
@@ -8642,7 +8645,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>